<commit_message>
feat: actualizar landing de Educacion Financiera a version responsiva universal (Habitos que Suman)
</commit_message>
<xml_diff>
--- a/public/Educacion-Financiera/Plantilla-Presupuesto-50-30-20-Rosed.xlsx
+++ b/public/Educacion-Financiera/Plantilla-Presupuesto-50-30-20-Rosed.xlsx
@@ -325,7 +325,7 @@
     <t>• 20% AHORRO: Tu yo del futuro (fondo de emergencia y fondo de retiro/largo plazo).</t>
   </si>
   <si>
-    <t>3. CLAVES PARA JOVENES DE 18 A 30 AÑOS:</t>
+    <t>3. CLAVES Y HÁBITOS QUE SUMAN:</t>
   </si>
   <si>
     <t>• Págate primero: Apenas cobres, transfiere tu 20% al ahorro antes de gastar.</t>
@@ -791,7 +791,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-963F-4CC4-B2B6-9F2BE9342FC4}"/>
+              <c16:uniqueId val="{00000000-7D96-4F43-8193-294182750922}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -844,7 +844,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-963F-4CC4-B2B6-9F2BE9342FC4}"/>
+              <c16:uniqueId val="{00000001-7D96-4F43-8193-294182750922}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -857,11 +857,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="405263248"/>
-        <c:axId val="405267824"/>
+        <c:axId val="1609889168"/>
+        <c:axId val="1609889584"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="405263248"/>
+        <c:axId val="1609889168"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -871,7 +871,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="405267824"/>
+        <c:crossAx val="1609889584"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -879,7 +879,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="405267824"/>
+        <c:axId val="1609889584"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -890,7 +890,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="405263248"/>
+        <c:crossAx val="1609889168"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1003,7 +1003,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-65C9-4714-BB27-4FE050768CC2}"/>
+              <c16:uniqueId val="{00000000-A637-4E85-A6DC-B938B76317AB}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1056,7 +1056,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-65C9-4714-BB27-4FE050768CC2}"/>
+              <c16:uniqueId val="{00000001-A637-4E85-A6DC-B938B76317AB}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1069,11 +1069,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:gapWidth val="150"/>
-        <c:axId val="405268240"/>
-        <c:axId val="405263664"/>
+        <c:axId val="1674786816"/>
+        <c:axId val="1674788064"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="405268240"/>
+        <c:axId val="1674786816"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1083,7 +1083,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="405263664"/>
+        <c:crossAx val="1674788064"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1091,7 +1091,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="405263664"/>
+        <c:axId val="1674788064"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1102,7 +1102,7 @@
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
-        <c:crossAx val="405268240"/>
+        <c:crossAx val="1674786816"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>